<commit_message>
feat: complete elearning enhancements and bugfixes
- Add ZIP download for submissions

- Add Angket approval flow for Admin and Tutor

- Implement flat-threaded nested replies for forum

- Fix RTE layout and input components
</commit_message>
<xml_diff>
--- a/public/templates/DAFTAR AGENDA TUTOR.xlsx
+++ b/public/templates/DAFTAR AGENDA TUTOR.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\PLCS\1PAND\PKBM\E-learning\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\web\production\E-learning\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE38427-8707-4176-B4B3-1DC8C08E384F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="750" windowWidth="29040" windowHeight="15570"/>
+    <workbookView xWindow="-120" yWindow="390" windowWidth="29040" windowHeight="15930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agenda Guru" sheetId="2" r:id="rId1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>YAYASAN MENUJU MAKMUR</t>
   </si>
@@ -41,32 +42,29 @@
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Wingdings"/>
         <charset val="2"/>
-        <color theme="1"/>
-        <sz val="10"/>
-        <scheme val="none"/>
       </rPr>
       <t>(</t>
     </r>
     <r>
       <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
-        <i val="1"/>
-        <color theme="1"/>
-        <sz val="10"/>
-        <scheme val="none"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
-        <color theme="1"/>
-        <sz val="10"/>
-        <scheme val="none"/>
       </rPr>
       <t xml:space="preserve"> 0811 2421 972</t>
     </r>
@@ -162,17 +160,14 @@
     <t>${namaTutor}</t>
   </si>
   <si>
-    <t>${nipTutor}</t>
-  </si>
-  <si>
-    <t>NIP.</t>
+    <t>NIP. ${nipTutor}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="34">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -435,109 +430,109 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.39994506668294322"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -603,25 +598,36 @@
     </fill>
   </fills>
   <borders count="15">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="medium">
         <color auto="1"/>
       </left>
+      <right/>
       <top style="medium">
         <color auto="1"/>
       </top>
       <bottom style="double">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="medium">
         <color auto="1"/>
       </top>
       <bottom style="double">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -630,6 +636,9 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -644,6 +653,7 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -652,9 +662,11 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -669,6 +681,7 @@
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -683,6 +696,7 @@
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="double">
@@ -697,26 +711,43 @@
       <bottom style="double">
         <color rgb="FF3F3F3F"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thick">
         <color theme="4"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thick">
         <color theme="4" tint="0.499984740745262"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.399975585192419"/>
+        <color theme="4" tint="0.39994506668294322"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -731,14 +762,18 @@
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="45">
@@ -788,7 +823,7 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -803,27 +838,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -831,22 +845,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -866,18 +871,52 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="45">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
-    <cellStyle name="Normal 22" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="3"/>
-    <cellStyle name="Note 2" xfId="4"/>
     <cellStyle name="20% - Accent1" xfId="5" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="6" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="7" builtinId="38" customBuiltin="1"/>
@@ -914,6 +953,11 @@
     <cellStyle name="Input" xfId="38" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="39" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="40" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 22" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Note 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Output" xfId="41" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Title" xfId="42" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="43" builtinId="25" customBuiltin="1"/>
@@ -923,7 +967,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505"/>
+          <bgColor theme="0" tint="-0.14993743705557422"/>
         </patternFill>
       </fill>
     </dxf>
@@ -937,6 +981,14 @@
       <color rgb="FF990099"/>
     </mruColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -957,7 +1009,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="40" name="Picture 39" descr="D:\PKBM\ADMINISTRASI LAIN\Logo PKBM.jpg"/>
+        <xdr:cNvPr id="40" name="Picture 39" descr="D:\PKBM\ADMINISTRASI LAIN\Logo PKBM.jpg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000028000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -971,13 +1029,15 @@
           <a:off x="10331824" y="78442"/>
           <a:ext cx="1064560" cy="868934"/>
         </a:xfrm>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
         <a:noFill/>
         <a:ln>
           <a:noFill/>
         </a:ln>
         <a:effectLst>
-          <a:reflection stA="50000" endA="275" endPos="40000" blurRad="6350" dist="101600" dir="5400000" sy="-100000" algn="bl" rotWithShape="0"/>
+          <a:reflection blurRad="6350" stA="50000" endA="275" endPos="40000" dist="101600" dir="5400000" sy="-100000" algn="bl" rotWithShape="0"/>
         </a:effectLst>
       </xdr:spPr>
     </xdr:pic>
@@ -998,7 +1058,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="41" name="Picture 40" descr="Description: D:\PKBM\logo pkbm menuju makmur.jpg"/>
+        <xdr:cNvPr id="41" name="Picture 40" descr="Description: D:\PKBM\logo pkbm menuju makmur.jpg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000029000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1014,7 +1080,9 @@
           <a:off x="119056" y="59669795"/>
           <a:ext cx="923010" cy="920846"/>
         </a:xfrm>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
         <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
@@ -1028,10 +1096,10 @@
   <a:themeElements>
     <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
-        <a:sysClr val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1163,7 +1231,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1187,11 +1254,10 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -1200,13 +1266,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1282,7 +1348,6 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1302,372 +1367,375 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" style="3" customWidth="1"/>
-    <col min="2" max="2" width="21.14063" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="8.140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="28.42578" style="5" customWidth="1"/>
-    <col min="5" max="5" width="32.71094" style="5" customWidth="1"/>
-    <col min="6" max="6" width="36.85547" style="5" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="36.85546875" style="5" customWidth="1"/>
     <col min="7" max="7" width="9" style="5" customWidth="1"/>
-    <col min="8" max="8" width="9.855469" style="5" customWidth="1"/>
-    <col min="9" max="9" width="21.42578" style="5" customWidth="1"/>
-    <col min="10" max="11" width="15.71094" style="3" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" style="5" customWidth="1"/>
+    <col min="10" max="11" width="15.7109375" style="3" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-    </row>
-    <row r="2" ht="27.75" customHeight="1">
-      <c r="A2" s="7" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+    </row>
+    <row r="2" spans="1:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="9" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="10" t="s">
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+    </row>
+    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-    </row>
-    <row r="5" thickBot="1" ht="15" customHeight="1">
-      <c r="A5" s="10" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+    </row>
+    <row r="5" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" thickBot="1" ht="15.75" customHeight="1">
-      <c r="A6" s="11" t="s">
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-    </row>
-    <row r="7" thickTop="1" ht="7.5" customHeight="1">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-    </row>
-    <row r="8" ht="7.5" customHeight="1">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="s">
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+    </row>
+    <row r="7" spans="1:9" ht="7.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="s">
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="s">
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17" t="s">
+      <c r="B13" s="25"/>
+      <c r="C13" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="s">
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17" t="s">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="17"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-    </row>
-    <row r="16" s="1" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A16" s="18" t="s">
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+    </row>
+    <row r="16" spans="1:9" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-    </row>
-    <row r="17" s="1" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19" t="s">
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+    </row>
+    <row r="17" spans="1:9" s="1" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="I17" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" s="2" customFormat="1" ht="27.95" customHeight="1">
-      <c r="A18" s="21" t="s">
+    <row r="18" spans="1:9" s="2" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="G18" s="23" t="s">
+      <c r="G18" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="H18" s="23" t="s">
+      <c r="H18" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="I18" s="23" t="s">
+      <c r="I18" s="13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="24" t="s">
+      <c r="H30" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="I30" s="24"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="25"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="24" t="s">
+      <c r="I30" s="19"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="15"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="I31" s="24"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="25"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="H32" s="24" t="s">
+      <c r="I31" s="19"/>
+    </row>
+    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="H32" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="I32" s="24"/>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="25"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="H33" s="24"/>
+      <c r="I32" s="19"/>
+    </row>
+    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="15"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="H33" s="14"/>
       <c r="I33" s="4"/>
     </row>
-    <row r="34">
-      <c r="A34" s="25"/>
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="25"/>
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="H35" s="28" t="s">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="15"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+    </row>
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="15"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+    </row>
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="15"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="18"/>
+      <c r="H36" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="I35" s="28"/>
-    </row>
-    <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="25"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="29"/>
-      <c r="H36" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="I36" s="3"/>
     </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="25"/>
-    </row>
-    <row r="38">
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
+    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="15"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="F16:F17"/>
+  <mergeCells count="20">
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="G16:I16"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="A11:I11"/>
@@ -1676,23 +1744,19 @@
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:I4"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="F16:F17"/>
   </mergeCells>
   <conditionalFormatting sqref="A18:I18">
-    <cfRule priority="1" dxfId="0" type="expression">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.7875" right="0.1965278" top="0.1965278" bottom="0.1965278" header="0" footer="0"/>
-  <pageSetup r:id="rId1" paperSize="0" orientation="portrait" scale="55"/>
+  <pageMargins left="0.78749999999999998" right="0.1965278" top="0.1965278" bottom="0.1965278" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="55" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>